<commit_message>
feat: implement news analyzer agent and add diagnostic scripts for data validation
</commit_message>
<xml_diff>
--- a/demo/newsapp/news_data/AAPL.xlsx
+++ b/demo/newsapp/news_data/AAPL.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,38 +413,63 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F90"/>
+  <dimension ref="A1:K90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>標題</t>
+          <t>title</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>日期</t>
+          <t>date</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>內容</t>
+          <t>content</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>連結</t>
+          <t>link</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>正負分析</t>
+          <t>source</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>來源</t>
+          <t>positive_negative_analysis</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>sentiment_score</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>market</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>confidence</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>impact_scope</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>reasoning_summary</t>
         </is>
       </c>
     </row>
@@ -471,12 +496,33 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -503,12 +549,33 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -535,12 +602,33 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -567,12 +655,33 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -599,12 +708,33 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -631,12 +761,33 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -663,12 +814,33 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>中性</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -695,12 +867,33 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>中性</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -727,12 +920,33 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -759,12 +973,33 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>中性</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -791,12 +1026,33 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -823,12 +1079,33 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -855,12 +1132,33 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -887,12 +1185,33 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -919,12 +1238,33 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -951,12 +1291,33 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>中性</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -983,12 +1344,33 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>中性</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -1015,12 +1397,33 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -1047,12 +1450,33 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>中性</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -1079,12 +1503,33 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -1111,12 +1556,33 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -1143,12 +1609,33 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -1175,12 +1662,33 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -1207,12 +1715,33 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -1239,12 +1768,33 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -1271,12 +1821,33 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>中性</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -1303,12 +1874,33 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G28" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -1335,12 +1927,33 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -1367,12 +1980,33 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -1399,12 +2033,33 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G31" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -1431,12 +2086,33 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G32" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>0</v>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -1463,12 +2139,33 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>中性</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G33" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>0</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -1495,12 +2192,33 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G34" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -1527,12 +2245,33 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>0</v>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -1559,12 +2298,33 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>0</v>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -1591,12 +2351,33 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G37" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>0</v>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -1623,12 +2404,33 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>0</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -1655,12 +2457,33 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>中性</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>0</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -1687,12 +2510,33 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>0</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -1719,12 +2563,33 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>0</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -1751,12 +2616,33 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>0</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -1783,12 +2669,33 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>中性</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>0</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -1815,12 +2722,33 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G44" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>0</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -1847,12 +2775,33 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>0</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -1879,12 +2828,33 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>0</v>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -1911,12 +2881,33 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>中性</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>0</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -1943,12 +2934,33 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>0</v>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -1975,12 +2987,33 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G49" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>0</v>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -2007,12 +3040,33 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G50" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
+        <v>0</v>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -2039,12 +3093,33 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G51" t="n">
+        <v>0</v>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I51" t="n">
+        <v>0</v>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -2071,12 +3146,33 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>中性</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G52" t="n">
+        <v>0</v>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
+        <v>0</v>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -2103,12 +3199,33 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G53" t="n">
+        <v>0</v>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I53" t="n">
+        <v>0</v>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -2135,12 +3252,33 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G54" t="n">
+        <v>0</v>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I54" t="n">
+        <v>0</v>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -2167,12 +3305,33 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G55" t="n">
+        <v>0</v>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I55" t="n">
+        <v>0</v>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -2199,12 +3358,33 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G56" t="n">
+        <v>0</v>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I56" t="n">
+        <v>0</v>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -2231,12 +3411,33 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>中性</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G57" t="n">
+        <v>0</v>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I57" t="n">
+        <v>0</v>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -2263,12 +3464,33 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G58" t="n">
+        <v>0</v>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I58" t="n">
+        <v>0</v>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -2295,12 +3517,33 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G59" t="n">
+        <v>0</v>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I59" t="n">
+        <v>0</v>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -2327,12 +3570,33 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G60" t="n">
+        <v>0</v>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I60" t="n">
+        <v>0</v>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -2359,12 +3623,33 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>中性</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G61" t="n">
+        <v>0</v>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I61" t="n">
+        <v>0</v>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -2391,12 +3676,33 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G62" t="n">
+        <v>0</v>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I62" t="n">
+        <v>0</v>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -2423,12 +3729,33 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G63" t="n">
+        <v>0</v>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I63" t="n">
+        <v>0</v>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -2455,12 +3782,33 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G64" t="n">
+        <v>0</v>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I64" t="n">
+        <v>0</v>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -2487,12 +3835,33 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G65" t="n">
+        <v>0</v>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I65" t="n">
+        <v>0</v>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -2519,12 +3888,33 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>中性</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G66" t="n">
+        <v>0</v>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I66" t="n">
+        <v>0</v>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -2551,12 +3941,33 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>中性</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G67" t="n">
+        <v>0</v>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I67" t="n">
+        <v>0</v>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -2583,12 +3994,33 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>中性</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G68" t="n">
+        <v>0</v>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I68" t="n">
+        <v>0</v>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -2615,12 +4047,33 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G69" t="n">
+        <v>0</v>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I69" t="n">
+        <v>0</v>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -2647,12 +4100,33 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G70" t="n">
+        <v>0</v>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I70" t="n">
+        <v>0</v>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -2679,12 +4153,33 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I71" t="n">
+        <v>0</v>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -2711,12 +4206,33 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G72" t="n">
+        <v>0</v>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I72" t="n">
+        <v>0</v>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -2743,12 +4259,33 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>中性</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G73" t="n">
+        <v>0</v>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I73" t="n">
+        <v>0</v>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -2775,12 +4312,33 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G74" t="n">
+        <v>0</v>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I74" t="n">
+        <v>0</v>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -2807,12 +4365,33 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G75" t="n">
+        <v>0</v>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I75" t="n">
+        <v>0</v>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -2839,12 +4418,33 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G76" t="n">
+        <v>0</v>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I76" t="n">
+        <v>0</v>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -2871,12 +4471,33 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G77" t="n">
+        <v>0</v>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I77" t="n">
+        <v>0</v>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -2903,12 +4524,33 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G78" t="n">
+        <v>0</v>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I78" t="n">
+        <v>0</v>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -2935,12 +4577,33 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G79" t="n">
+        <v>0</v>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I79" t="n">
+        <v>0</v>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -2967,12 +4630,33 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>中性</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G80" t="n">
+        <v>0</v>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I80" t="n">
+        <v>0</v>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -2999,12 +4683,33 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>中性</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G81" t="n">
+        <v>0</v>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I81" t="n">
+        <v>0</v>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -3031,12 +4736,33 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G82" t="n">
+        <v>0</v>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I82" t="n">
+        <v>0</v>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -3063,12 +4789,33 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>中性</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G83" t="n">
+        <v>0</v>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I83" t="n">
+        <v>0</v>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -3095,12 +4842,33 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G84" t="n">
+        <v>0</v>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I84" t="n">
+        <v>0</v>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -3127,12 +4895,33 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G85" t="n">
+        <v>0</v>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I85" t="n">
+        <v>0</v>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -3159,12 +4948,33 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>中性</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G86" t="n">
+        <v>0</v>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I86" t="n">
+        <v>0</v>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -3191,12 +5001,33 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G87" t="n">
+        <v>0</v>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I87" t="n">
+        <v>0</v>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -3223,12 +5054,33 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G88" t="n">
+        <v>0</v>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I88" t="n">
+        <v>0</v>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -3255,12 +5107,33 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G89" t="n">
+        <v>0</v>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I89" t="n">
+        <v>0</v>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>
@@ -3287,12 +5160,33 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>正面</t>
+          <t>鉅亨網-美股-AAPL</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>鉅亨網-美股-AAPL</t>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="G90" t="n">
+        <v>0</v>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="I90" t="n">
+        <v>0</v>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>短期</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>Agent 呼叫失敗，請檢查 API Key 或網路連線。</t>
         </is>
       </c>
     </row>

</xml_diff>